<commit_message>
Position outreach pipeline for AI portfolio
</commit_message>
<xml_diff>
--- a/outputs/outreach_pipeline_masked.xlsx
+++ b/outputs/outreach_pipeline_masked.xlsx
@@ -3398,15 +3398,16 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>{{Компания}} и холодные письма</t>
+          <t>{{Компания}} and outbound email</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>{{Имя}}, привет.
+          <t>{{Имя}}, hello.
 {{персонализация}}
-Мы запускаем холодный email для B2B: база, письма, домены и первые ответы. Для {{Компания}} я бы начал с короткого пилота на 2-3 сегмента.
-Хотите, покажу, как это может выглядеть у вас?</t>
+We help B2B teams test outbound email without turning it into a large, risky campaign from day one: segment, offer, sequence, domain setup, and reply tracking.
+For {{Компания}}, I would start with a small pilot: 2-3 segments, a separate offer for each, and clear reply metrics before scaling.
+Would it be useful if I showed what that pilot could look like for your market?</t>
         </is>
       </c>
     </row>
@@ -3418,14 +3419,15 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Re: {{Компания}} и холодные письма</t>
+          <t>Re: {{Компания}} and outbound email</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>{{Имя}}, вдогонку коротко.
-Часто проблема не в канале, а в запуске: база собрана не по ICP, домен холодный, письма читаются как спам.
-Если интересно, давайте 15 минут, покажу механику запуска.</t>
+          <t>{{Имя}}, quick follow-up.
+When cold email does not work, the problem is often not the channel itself. Usually the list is too broad, the domain is cold, or the email reads like a generic template.
+The safer version is to test in small batches: validate the segment, keep the copy specific, track replies, and only then scale.
+If this is relevant, I can share a short outline for a pilot campaign.</t>
         </is>
       </c>
     </row>
@@ -3437,14 +3439,14 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Re: {{Компания}} и холодные письма</t>
+          <t>Re: {{Компания}} and outbound email</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>{{Имя}}, всё, последнее.
-Холодный email нормально работает, когда это серия маленьких тестов: сегмент, оффер, письмо, ответ.
-Если тема всплывёт позже, ответьте на это письмо. Договоримся.</t>
+          <t>{{Имя}}, last note from me.
+Cold email works best when it is treated as a series of small tests: segment, offer, message, reply quality. That also keeps the risk low before a bigger rollout.
+If this becomes relevant later, you can reply to this email and I will send over a compact campaign outline.</t>
         </is>
       </c>
     </row>
@@ -3459,7 +3461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3536,6 +3538,18 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Agent workflow</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>documented in docs/agent_workflow.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>